<commit_message>
Aktualizace dat z webové aplikace
</commit_message>
<xml_diff>
--- a/prohlidky.xlsx
+++ b/prohlidky.xlsx
@@ -1035,23 +1035,23 @@
         </is>
       </c>
       <c r="B21" s="1" t="n">
-        <v>46174</v>
+        <v>46277</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>P-2</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>46368</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
           <t>P-3</t>
         </is>
       </c>
-      <c r="D21" s="1" t="n">
-        <v>46266</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>P-2</t>
-        </is>
-      </c>
       <c r="F21" s="1" t="n">
-        <v>46266</v>
+        <v>47008</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>

</xml_diff>